<commit_message>
Conteúdo: modelo de newsletter FSA e planilha com camadas e regra do carrossel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -506,202 +506,274 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>VISÃO</t>
+          <t>AS CAMADAS (ler primeiro)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
+          <t>O PRINCIPAL DA SEMANA é transformar seguidor em base (e-mail). O número que mais importa: e-mails novos + cliques na newsletter.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>RESPONSÁVEL</t>
+          <t>CAMADA 1 · O CENTRO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
+          <t>Tema da semana (vem da live) → NEWSLETTER. É o produto da semana e o que mantém a base quente.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>QUEM APARECE</t>
+          <t>CAMADA 2 · A PONTE</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>Criativo de captura ("comenta e recebe"). Leva a pessoa do Instagram para dentro da base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>O CENTRO DA SEMANA</t>
+          <t>CAMADA 3 · O COMBUSTÍVEL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>Reels e carrosséis. Atraem gente nova e aquecem quem já segue. Uns 3 por semana no tema da semana; o resto nos assuntos fixos ligados às formações (para o perfil não ficar repetitivo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ENTREGAS DA SEMANA</t>
+          <t>CARROSSEL DA NEWSLETTER</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter. Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
+          <t>NUNCA abrir com "o tema da newsletter desta semana". A capa é a ideia mais surpreendente que está DENTRO da newsletter, algo que quebra a cabeça e faz rolar. Só no último slide a pessoa descobre que aquilo é um pedaço da newsletter: "Isso saiu na nossa newsletter desta semana. Quer receber as próximas? Comenta NEWS."</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+          <t>VISÃO</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>RESPONSÁVEL</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>QUEM APARECE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>O CENTRO DA SEMANA</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ENTREGAS DA SEMANA</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter. Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>MATERIAL DE CAPTURA</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico validado pelo professor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>ROTINA (D = dia da live)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>D+1: transcrição (Descript) e rascunho da newsletter. D+2: revisão técnica do professor da live + pacote da semana para a Gisele aprovar. D+3: newsletter enviada. D+3 a D+6: reels, carrosséis e captura publicados. Toda semana: preencher abas 4 e 5 (15 min).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>D+1: transcrição (Descript) e rascunho da newsletter. D+2: pacote da semana para a Gisele aprovar. D+3: newsletter enviada. D+3 a D+6: reels, carrosséis e captura publicados. Toda semana: preencher abas 4 e 5 (15 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>IMAGENS (responsabilidade dela)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Todo roteiro e carrossel sai com as imagens escolhidas, não só o texto. Imagem REAL, nunca de IA: professores, aulas, bastidores, prova (depoimentos e prints de alunos), e imagem daquilo que se está falando (o exame, o suplemento, o alimento). Muita imagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>BANCO DE IMAGENS</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Manter uma pasta no Drive organizada por tema (professores, aulas, bastidores, prova, exames, alimentos). Quando faltar imagem de um tema, pedir foto ao professor ou à equipe com antecedência.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>AUTORIZAÇÃO DE IMAGEM</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>APROVAÇÃO</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Tudo passa pela Gisele antes de sair, em LOTE: uma vez por semana, o pacote inteiro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>PRIORIDADE SE O TEMPO APERTAR</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>A META É RESULTADO</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>BANCO DE IMAGENS</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ARTE COM IA</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Pode usar IA para montar a arte do carrossel (layout, tipografia, cores). As FOTOS dentro da arte são reais, nunca geradas por IA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>AUTORIZAÇÃO DE IMAGEM</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>APROVAÇÃO</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Tudo passa pela Gisele antes de sair, em LOTE: uma vez por semana, o pacote inteiro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>A META É RESULTADO</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>TODA SEMANA, 3 LINHAS</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>O que funcionou. O que não funcionou. O que vou testar na semana que vem. (aba 5)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>REGRAS QUE NÃO MUDAM</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>BASE DE E-MAIL</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Reaquecer em ordem: semanas 1 e 2 só para quem abriu ou clicou nos últimos 6 meses; semana 3 campanha de reativação para os parados; depois tirar do envio quem não abre há 12 meses. Spam acima de 0,1%: parar e corrigir.</t>
         </is>
@@ -3244,7 +3316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3422,7 +3494,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>FATOS: todo dado técnico tem fonte e foi validado pelo professor.</t>
+          <t>FATOS: todo dado técnico vem do material da FSA (live, aula) ou tem fonte.</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3506,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>REGRAS: sem promessa de cura ou resultado garantido; dentro das regras do conselho.</t>
+          <t>CARROSSEL DA NEWSLETTER: a capa NÃO diz "tema da newsletter". Abre com a ideia que quebra a cabeça; a newsletter só aparece no último slide.</t>
         </is>
       </c>
     </row>
@@ -3445,6 +3517,18 @@
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>REGRAS: sem promessa de cura ou resultado garantido; dentro das regras do conselho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>CAMPANHA: se fala de oferta, diz exatamente o que a página de destino diz (mesma frase, número, prazo).</t>
         </is>
@@ -3509,7 +3593,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Validado pelo professor?</t>
+          <t>Tirado de qual material?</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Planilha: regra da arte do carrossel (Claude monta, fotos enviadas por ela)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -686,12 +686,12 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ARTE COM IA</t>
+          <t>ARTE DO CARROSSEL</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Pode usar IA para montar a arte do carrossel (layout, tipografia, cores). As FOTOS dentro da arte são reais, nunca geradas por IA.</t>
+          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilha: explica os 3 níveis de medição (entregas, KPIs, OKR)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -563,217 +563,241 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="75" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>VISÃO</t>
+          <t>COMO SOMOS MEDIDOS (3 níveis)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
+          <t>1) TODA SEMANA, ENTREGAS (aba 3): fiz o que combinei? Meta 100%. 2) TODA SEMANA, KPIs (aba 5): os números que mostram se a operação está saudável (seguidores novos, engajados, e-mails novos, cliques). Eu trago e comparo com a semana anterior. 3) TODO MÊS, OKR (aba 2): a meta de RESULTADO do mês. É o que diz se o trabalho trouxe resultado. E em cada peça, o PLACAR (aba 4): gancho, retenção e conversão de cada reel e carrossel.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RESPONSÁVEL</t>
+          <t>OKR x KPI</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
+          <t>OKR é o que queremos MUDAR no mês (crescer a base, aumentar cliques). KPI é o que não podemos deixar PIORAR toda semana. OKR muda a cada mês; KPI é sempre o mesmo painel.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>QUEM APARECE</t>
+          <t>VISÃO</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
+          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>O CENTRO DA SEMANA</t>
+          <t>RESPONSÁVEL</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
+          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>QUEM APARECE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>O CENTRO DA SEMANA</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>ENTREGAS DA SEMANA</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>5 roteiros de reels + 4 carrosséis + 1 newsletter. Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>CRIATIVO DE CAPTURA (rodízio)</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>MATERIAL DE CAPTURA</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ROTINA (D = dia da live)</t>
+          <t>CRIATIVO DE CAPTURA (rodízio)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>D+1: transcrição (Descript) e rascunho da newsletter. D+2: pacote da semana para a Gisele aprovar. D+3: newsletter enviada. D+3 a D+6: reels, carrosséis e captura publicados. Toda semana: preencher abas 4 e 5 (15 min).</t>
+          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>MATERIAL DE CAPTURA</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ROTINA (D = dia da live)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>D+1: transcrição (Descript) e rascunho da newsletter. D+2: pacote da semana para a Gisele aprovar. D+3: newsletter enviada. D+3 a D+6: reels, carrosséis e captura publicados. Toda semana: preencher abas 4 e 5 (15 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>IMAGENS (responsabilidade dela)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Todo roteiro e carrossel sai com as imagens escolhidas, não só o texto. Imagem REAL, nunca de IA: professores, aulas, bastidores, prova (depoimentos e prints de alunos), e imagem daquilo que se está falando (o exame, o suplemento, o alimento). Muita imagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>BANCO DE IMAGENS</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>ARTE DO CARROSSEL</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AUTORIZAÇÃO DE IMAGEM</t>
+          <t>BANCO DE IMAGENS</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
+          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>APROVAÇÃO</t>
+          <t>ARTE DO CARROSSEL</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Tudo passa pela Gisele antes de sair, em LOTE: uma vez por semana, o pacote inteiro.</t>
+          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+          <t>AUTORIZAÇÃO DE IMAGEM</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels</t>
+          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>A META É RESULTADO</t>
+          <t>APROVAÇÃO</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+          <t>Tudo passa pela Gisele antes de sair, em LOTE: uma vez por semana, o pacote inteiro.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>A META É RESULTADO</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>TODA SEMANA, 3 LINHAS</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>O que funcionou. O que não funcionou. O que vou testar na semana que vem. (aba 5)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>REGRAS QUE NÃO MUDAM</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>BASE DE E-MAIL</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Reaquecer em ordem: semanas 1 e 2 só para quem abriu ou clicou nos últimos 6 meses; semana 3 campanha de reativação para os parados; depois tirar do envio quem não abre há 12 meses. Spam acima de 0,1%: parar e corrigir.</t>
         </is>

</xml_diff>

<commit_message>
Roteiro de apresentação para a gerente; entrega semanal na sexta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -671,7 +671,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="45" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>ROTINA (D = dia da live)</t>
@@ -679,7 +679,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>D+1: transcrição (Descript) e rascunho da newsletter. D+2: pacote da semana para a Gisele aprovar. D+3: newsletter enviada. D+3 a D+6: reels, carrosséis e captura publicados. Toda semana: preencher abas 4 e 5 (15 min).</t>
+          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tudo passa pela Gisele antes de sair, em LOTE: uma vez por semana, o pacote inteiro.</t>
+          <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plano de conteúdo: YouTube (Shorts + live da semana) na planilha e no roteiro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Reels e carrosséis. Atraem gente nova e aquecem quem já segue. Uns 3 por semana no tema da semana; o resto nos assuntos fixos ligados às formações (para o perfil não ficar repetitivo).</t>
+          <t>Reels, carrosséis e YouTube. Atraem gente nova e aquecem quem já segue. Uns 3 por semana no tema da semana; o resto nos assuntos fixos ligados às formações (para o perfil não ficar repetitivo).</t>
         </is>
       </c>
     </row>
@@ -643,161 +643,197 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter. Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
+          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter + YouTube (5 Shorts + a live da semana). Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+          <t>YOUTUBE: SHORTS</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+          <t>Os 5 reels da semana sobem também como Shorts no YouTube. Sem roteiro novo: é repostar, com título próprio para o YouTube.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MATERIAL DE CAPTURA</t>
+          <t>YOUTUBE: A LIVE DA SEMANA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
+          <t>A gravação da live sobe no YouTube toda semana. O trabalho dela: título forte (com a palavra que a pessoa buscaria no Google), capa com foto real e texto grande, descrição com o resumo, os momentos principais e o link da newsletter. Tempo: uns 30 minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ROTINA (D = dia da live)</t>
+          <t>YOUTUBE: O PAPEL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
+          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. No futuro, se der resultado, pode entrar 1 vídeo roteirizado por semana; nesse caso, sai 2 reels para abrir espaço.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>MATERIAL DE CAPTURA</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ROTINA (D = dia da live)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>IMAGENS (responsabilidade dela)</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Todo roteiro e carrossel sai com as imagens escolhidas, não só o texto. Imagem REAL, nunca de IA: professores, aulas, bastidores, prova (depoimentos e prints de alunos), e imagem daquilo que se está falando (o exame, o suplemento, o alimento). Muita imagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>BANCO DE IMAGENS</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>ARTE DO CARROSSEL</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>AUTORIZAÇÃO DE IMAGEM</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>APROVAÇÃO</t>
+          <t>BANCO DE IMAGENS</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
+          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+          <t>ARTE DO CARROSSEL</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels</t>
+          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>A META É RESULTADO</t>
+          <t>AUTORIZAÇÃO DE IMAGEM</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>APROVAÇÃO</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels  5) Live no YouTube  6) Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>A META É RESULTADO</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>TODA SEMANA, 3 LINHAS</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>O que funcionou. O que não funcionou. O que vou testar na semana que vem. (aba 5)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>REGRAS QUE NÃO MUDAM</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>BASE DE E-MAIL</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Reaquecer em ordem: semanas 1 e 2 só para quem abriu ou clicou nos últimos 6 meses; semana 3 campanha de reativação para os parados; depois tirar do envio quem não abre há 12 meses. Spam acima de 0,1%: parar e corrigir.</t>
         </is>
@@ -1025,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1037,6 +1073,8 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1090,6 +1128,16 @@
       <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Observação</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Shorts no YouTube (meta 5)</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Live no YouTube (1)</t>
         </is>
       </c>
     </row>
@@ -1101,11 +1149,13 @@
       <c r="E4" s="9" t="n"/>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="12">
-        <f>IF(A4="","",(MIN(B4,5)+MIN(C4,4)+MIN(D4,1)+MIN(E4,1))/11)</f>
+        <f>IF(A4="","",(MIN(B4,5)+MIN(C4,4)+MIN(D4,1)+MIN(E4,1)+MIN(J4,5)+MIN(K4,1))/17)</f>
         <v/>
       </c>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
+      <c r="J4" s="9" t="n"/>
+      <c r="K4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -1115,11 +1165,13 @@
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="9" t="n"/>
       <c r="G5" s="12">
-        <f>IF(A5="","",(MIN(B5,5)+MIN(C5,4)+MIN(D5,1)+MIN(E5,1))/11)</f>
+        <f>IF(A5="","",(MIN(B5,5)+MIN(C5,4)+MIN(D5,1)+MIN(E5,1)+MIN(J5,5)+MIN(K5,1))/17)</f>
         <v/>
       </c>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="9" t="n"/>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -1129,11 +1181,13 @@
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="12">
-        <f>IF(A6="","",(MIN(B6,5)+MIN(C6,4)+MIN(D6,1)+MIN(E6,1))/11)</f>
+        <f>IF(A6="","",(MIN(B6,5)+MIN(C6,4)+MIN(D6,1)+MIN(E6,1)+MIN(J6,5)+MIN(K6,1))/17)</f>
         <v/>
       </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -1143,11 +1197,13 @@
       <c r="E7" s="9" t="n"/>
       <c r="F7" s="9" t="n"/>
       <c r="G7" s="12">
-        <f>IF(A7="","",(MIN(B7,5)+MIN(C7,4)+MIN(D7,1)+MIN(E7,1))/11)</f>
+        <f>IF(A7="","",(MIN(B7,5)+MIN(C7,4)+MIN(D7,1)+MIN(E7,1)+MIN(J7,5)+MIN(K7,1))/17)</f>
         <v/>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -1157,11 +1213,13 @@
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="9" t="n"/>
       <c r="G8" s="12">
-        <f>IF(A8="","",(MIN(B8,5)+MIN(C8,4)+MIN(D8,1)+MIN(E8,1))/11)</f>
+        <f>IF(A8="","",(MIN(B8,5)+MIN(C8,4)+MIN(D8,1)+MIN(E8,1)+MIN(J8,5)+MIN(K8,1))/17)</f>
         <v/>
       </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -1171,11 +1229,13 @@
       <c r="E9" s="9" t="n"/>
       <c r="F9" s="9" t="n"/>
       <c r="G9" s="12">
-        <f>IF(A9="","",(MIN(B9,5)+MIN(C9,4)+MIN(D9,1)+MIN(E9,1))/11)</f>
+        <f>IF(A9="","",(MIN(B9,5)+MIN(C9,4)+MIN(D9,1)+MIN(E9,1)+MIN(J9,5)+MIN(K9,1))/17)</f>
         <v/>
       </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -1185,11 +1245,13 @@
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
       <c r="G10" s="12">
-        <f>IF(A10="","",(MIN(B10,5)+MIN(C10,4)+MIN(D10,1)+MIN(E10,1))/11)</f>
+        <f>IF(A10="","",(MIN(B10,5)+MIN(C10,4)+MIN(D10,1)+MIN(E10,1)+MIN(J10,5)+MIN(K10,1))/17)</f>
         <v/>
       </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -1199,11 +1261,13 @@
       <c r="E11" s="9" t="n"/>
       <c r="F11" s="9" t="n"/>
       <c r="G11" s="12">
-        <f>IF(A11="","",(MIN(B11,5)+MIN(C11,4)+MIN(D11,1)+MIN(E11,1))/11)</f>
+        <f>IF(A11="","",(MIN(B11,5)+MIN(C11,4)+MIN(D11,1)+MIN(E11,1)+MIN(J11,5)+MIN(K11,1))/17)</f>
         <v/>
       </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -1213,11 +1277,13 @@
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="9" t="n"/>
       <c r="G12" s="12">
-        <f>IF(A12="","",(MIN(B12,5)+MIN(C12,4)+MIN(D12,1)+MIN(E12,1))/11)</f>
+        <f>IF(A12="","",(MIN(B12,5)+MIN(C12,4)+MIN(D12,1)+MIN(E12,1)+MIN(J12,5)+MIN(K12,1))/17)</f>
         <v/>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -1227,11 +1293,13 @@
       <c r="E13" s="9" t="n"/>
       <c r="F13" s="9" t="n"/>
       <c r="G13" s="12">
-        <f>IF(A13="","",(MIN(B13,5)+MIN(C13,4)+MIN(D13,1)+MIN(E13,1))/11)</f>
+        <f>IF(A13="","",(MIN(B13,5)+MIN(C13,4)+MIN(D13,1)+MIN(E13,1)+MIN(J13,5)+MIN(K13,1))/17)</f>
         <v/>
       </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -1241,11 +1309,13 @@
       <c r="E14" s="9" t="n"/>
       <c r="F14" s="9" t="n"/>
       <c r="G14" s="12">
-        <f>IF(A14="","",(MIN(B14,5)+MIN(C14,4)+MIN(D14,1)+MIN(E14,1))/11)</f>
+        <f>IF(A14="","",(MIN(B14,5)+MIN(C14,4)+MIN(D14,1)+MIN(E14,1)+MIN(J14,5)+MIN(K14,1))/17)</f>
         <v/>
       </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -1255,11 +1325,13 @@
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="9" t="n"/>
       <c r="G15" s="12">
-        <f>IF(A15="","",(MIN(B15,5)+MIN(C15,4)+MIN(D15,1)+MIN(E15,1))/11)</f>
+        <f>IF(A15="","",(MIN(B15,5)+MIN(C15,4)+MIN(D15,1)+MIN(E15,1)+MIN(J15,5)+MIN(K15,1))/17)</f>
         <v/>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -1269,11 +1341,13 @@
       <c r="E16" s="9" t="n"/>
       <c r="F16" s="9" t="n"/>
       <c r="G16" s="12">
-        <f>IF(A16="","",(MIN(B16,5)+MIN(C16,4)+MIN(D16,1)+MIN(E16,1))/11)</f>
+        <f>IF(A16="","",(MIN(B16,5)+MIN(C16,4)+MIN(D16,1)+MIN(E16,1)+MIN(J16,5)+MIN(K16,1))/17)</f>
         <v/>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2951,7 +3025,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Reel,Carrossel,Newsletter"</formula1>
+      <formula1>"Reel,Carrossel,Newsletter,Short,Live YouTube"</formula1>
     </dataValidation>
     <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Gabriel,Liliane,Outro"</formula1>
@@ -2970,7 +3044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2984,9 +3058,13 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="34" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3054,15 +3132,35 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
+          <t>YouTube: inscritos novos</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>YouTube: visualizações</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>YouTube: horas assistidas</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>YouTube: cliques no link da newsletter</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
           <t>O que funcionou</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>O que não funcionou</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>O que vou testar na semana que vem</t>
         </is>
@@ -3083,9 +3181,13 @@
         <f>IF(A4="","",COUNTIFS('4. Placar por peça'!A:A,A4,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A4,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L4" s="17" t="n"/>
-      <c r="M4" s="17" t="n"/>
-      <c r="N4" s="17" t="n"/>
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="n"/>
+      <c r="N4" s="9" t="n"/>
+      <c r="O4" s="9" t="n"/>
+      <c r="P4" s="17" t="n"/>
+      <c r="Q4" s="17" t="n"/>
+      <c r="R4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -3102,9 +3204,13 @@
         <f>IF(A5="","",COUNTIFS('4. Placar por peça'!A:A,A5,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A5,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="n"/>
+      <c r="O5" s="9" t="n"/>
+      <c r="P5" s="17" t="n"/>
+      <c r="Q5" s="17" t="n"/>
+      <c r="R5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -3121,9 +3227,13 @@
         <f>IF(A6="","",COUNTIFS('4. Placar por peça'!A:A,A6,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A6,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="17" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9" t="n"/>
+      <c r="O6" s="9" t="n"/>
+      <c r="P6" s="17" t="n"/>
+      <c r="Q6" s="17" t="n"/>
+      <c r="R6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -3140,9 +3250,13 @@
         <f>IF(A7="","",COUNTIFS('4. Placar por peça'!A:A,A7,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A7,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n"/>
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="9" t="n"/>
+      <c r="N7" s="9" t="n"/>
+      <c r="O7" s="9" t="n"/>
+      <c r="P7" s="17" t="n"/>
+      <c r="Q7" s="17" t="n"/>
+      <c r="R7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -3159,9 +3273,13 @@
         <f>IF(A8="","",COUNTIFS('4. Placar por peça'!A:A,A8,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A8,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="17" t="n"/>
-      <c r="N8" s="17" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
+      <c r="O8" s="9" t="n"/>
+      <c r="P8" s="17" t="n"/>
+      <c r="Q8" s="17" t="n"/>
+      <c r="R8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -3178,9 +3296,13 @@
         <f>IF(A9="","",COUNTIFS('4. Placar por peça'!A:A,A9,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A9,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="17" t="n"/>
-      <c r="N9" s="17" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="9" t="n"/>
+      <c r="O9" s="9" t="n"/>
+      <c r="P9" s="17" t="n"/>
+      <c r="Q9" s="17" t="n"/>
+      <c r="R9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -3197,9 +3319,13 @@
         <f>IF(A10="","",COUNTIFS('4. Placar por peça'!A:A,A10,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A10,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9" t="n"/>
+      <c r="O10" s="9" t="n"/>
+      <c r="P10" s="17" t="n"/>
+      <c r="Q10" s="17" t="n"/>
+      <c r="R10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -3216,9 +3342,13 @@
         <f>IF(A11="","",COUNTIFS('4. Placar por peça'!A:A,A11,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A11,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="17" t="n"/>
-      <c r="N11" s="17" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
+      <c r="O11" s="9" t="n"/>
+      <c r="P11" s="17" t="n"/>
+      <c r="Q11" s="17" t="n"/>
+      <c r="R11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -3235,9 +3365,13 @@
         <f>IF(A12="","",COUNTIFS('4. Placar por peça'!A:A,A12,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A12,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="17" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="n"/>
+      <c r="O12" s="9" t="n"/>
+      <c r="P12" s="17" t="n"/>
+      <c r="Q12" s="17" t="n"/>
+      <c r="R12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -3254,9 +3388,13 @@
         <f>IF(A13="","",COUNTIFS('4. Placar por peça'!A:A,A13,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A13,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="17" t="n"/>
-      <c r="N13" s="17" t="n"/>
+      <c r="L13" s="9" t="n"/>
+      <c r="M13" s="9" t="n"/>
+      <c r="N13" s="9" t="n"/>
+      <c r="O13" s="9" t="n"/>
+      <c r="P13" s="17" t="n"/>
+      <c r="Q13" s="17" t="n"/>
+      <c r="R13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -3273,9 +3411,13 @@
         <f>IF(A14="","",COUNTIFS('4. Placar por peça'!A:A,A14,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A14,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L14" s="17" t="n"/>
-      <c r="M14" s="17" t="n"/>
-      <c r="N14" s="17" t="n"/>
+      <c r="L14" s="9" t="n"/>
+      <c r="M14" s="9" t="n"/>
+      <c r="N14" s="9" t="n"/>
+      <c r="O14" s="9" t="n"/>
+      <c r="P14" s="17" t="n"/>
+      <c r="Q14" s="17" t="n"/>
+      <c r="R14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -3292,9 +3434,13 @@
         <f>IF(A15="","",COUNTIFS('4. Placar por peça'!A:A,A15,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A15,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L15" s="17" t="n"/>
-      <c r="M15" s="17" t="n"/>
-      <c r="N15" s="17" t="n"/>
+      <c r="L15" s="9" t="n"/>
+      <c r="M15" s="9" t="n"/>
+      <c r="N15" s="9" t="n"/>
+      <c r="O15" s="9" t="n"/>
+      <c r="P15" s="17" t="n"/>
+      <c r="Q15" s="17" t="n"/>
+      <c r="R15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -3311,9 +3457,13 @@
         <f>IF(A16="","",COUNTIFS('4. Placar por peça'!A:A,A16,'4. Placar por peça'!C:C,"Reel",'4. Placar por peça'!V:V,"Sim")&amp;" de "&amp;COUNTIFS('4. Placar por peça'!A:A,A16,'4. Placar por peça'!C:C,"Reel"))</f>
         <v/>
       </c>
-      <c r="L16" s="17" t="n"/>
-      <c r="M16" s="17" t="n"/>
-      <c r="N16" s="17" t="n"/>
+      <c r="L16" s="9" t="n"/>
+      <c r="M16" s="9" t="n"/>
+      <c r="N16" s="9" t="n"/>
+      <c r="O16" s="9" t="n"/>
+      <c r="P16" s="17" t="n"/>
+      <c r="Q16" s="17" t="n"/>
+      <c r="R16" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3340,7 +3490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3553,6 +3703,18 @@
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>YOUTUBE (live): título com a palavra que a pessoa buscaria, capa com foto real e texto grande, descrição com resumo, momentos principais e link da newsletter, comentário fixado com o link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>CAMPANHA: se fala de oferta, diz exatamente o que a página de destino diz (mesma frase, número, prazo).</t>
         </is>

</xml_diff>

<commit_message>
YouTube: vídeo roteirizado semanal e regras de thumb na planilha e no roteiro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -635,7 +635,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>ENTREGAS DA SEMANA</t>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter + YouTube (5 Shorts + a live da semana). Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
+          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter + YouTube (5 Shorts + 1 vídeo roteirizado + a live da semana). Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
         </is>
       </c>
     </row>
@@ -671,169 +671,193 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="45" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>YOUTUBE: O PAPEL</t>
+          <t>YOUTUBE: VÍDEO ROTEIRIZADO</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. No futuro, se der resultado, pode entrar 1 vídeo roteirizado por semana; nesse caso, sai 2 reels para abrir espaço.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
+          <t>1 por semana, de 8 a 15 minutos, gravado pelo Gabriel ou pela Liliane. Usa o MESMO tema da newsletter da semana, mais aprofundado: a pesquisa já está feita, então o trabalho é o roteiro. Estrutura: gancho nos primeiros 30 segundos (a promessa do vídeo), desenvolvimento em blocos, caso prático, chamada para a newsletter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="75" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+          <t>YOUTUBE: THUMB (CAPA)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+          <t>Toda thumb tem ROSTO, nunca só nome ou texto. Rosto grande, com expressão que chama atenção (surpresa, dúvida, preocupação, apontando). Foto real do professor, feita para a thumb. Até 4 palavras em letra grande, que completam o título sem repetir. Flecha ou círculo apontando para o elemento principal (o exame, o alimento, o número). Contraste forte. Testar se dá para ler no tamanho de celular.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MATERIAL DE CAPTURA</t>
+          <t>YOUTUBE: O PAPEL</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1">
+          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. O número que mostra se a thumb funciona é a TAXA DE CLIQUES (CTR) das impressões, no YouTube Studio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ROTINA (D = dia da live)</t>
+          <t>CRIATIVO DE CAPTURA (rodízio)</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
+          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>MATERIAL DE CAPTURA</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ROTINA (D = dia da live)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>IMAGENS (responsabilidade dela)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Todo roteiro e carrossel sai com as imagens escolhidas, não só o texto. Imagem REAL, nunca de IA: professores, aulas, bastidores, prova (depoimentos e prints de alunos), e imagem daquilo que se está falando (o exame, o suplemento, o alimento). Muita imagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>BANCO DE IMAGENS</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>ARTE DO CARROSSEL</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>AUTORIZAÇÃO DE IMAGEM</t>
+          <t>BANCO DE IMAGENS</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
+          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>APROVAÇÃO</t>
+          <t>ARTE DO CARROSSEL</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
+          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+          <t>AUTORIZAÇÃO DE IMAGEM</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>1) Newsletter  2) Criativo de captura  3) Carrosséis  4) Reels  5) Live no YouTube  6) Shorts</t>
+          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>A META É RESULTADO</t>
+          <t>APROVAÇÃO</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+          <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>PRIORIDADE SE O TEMPO APERTAR</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>1) Newsletter  2) Criativo de captura  3) Vídeo roteirizado do YouTube  4) Carrosséis  5) Reels  6) Live no YouTube  7) Shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>A META É RESULTADO</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>TODA SEMANA, 3 LINHAS</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>O que funcionou. O que não funcionou. O que vou testar na semana que vem. (aba 5)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>REGRAS QUE NÃO MUDAM</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>BASE DE E-MAIL</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Reaquecer em ordem: semanas 1 e 2 só para quem abriu ou clicou nos últimos 6 meses; semana 3 campanha de reativação para os parados; depois tirar do envio quem não abre há 12 meses. Spam acima de 0,1%: parar e corrigir.</t>
         </is>
@@ -1061,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1075,6 +1099,7 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1138,6 +1163,11 @@
       <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Live no YouTube (1)</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Vídeo roteirizado no YouTube (1)</t>
         </is>
       </c>
     </row>
@@ -1149,13 +1179,14 @@
       <c r="E4" s="9" t="n"/>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="12">
-        <f>IF(A4="","",(MIN(B4,5)+MIN(C4,4)+MIN(D4,1)+MIN(E4,1)+MIN(J4,5)+MIN(K4,1))/17)</f>
+        <f>IF(A4="","",(MIN(B4,5)+MIN(C4,4)+MIN(D4,1)+MIN(E4,1)+MIN(J4,5)+MIN(K4,1)+MIN(L4,1))/18)</f>
         <v/>
       </c>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
       <c r="J4" s="9" t="n"/>
       <c r="K4" s="9" t="n"/>
+      <c r="L4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -1165,13 +1196,14 @@
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="9" t="n"/>
       <c r="G5" s="12">
-        <f>IF(A5="","",(MIN(B5,5)+MIN(C5,4)+MIN(D5,1)+MIN(E5,1)+MIN(J5,5)+MIN(K5,1))/17)</f>
+        <f>IF(A5="","",(MIN(B5,5)+MIN(C5,4)+MIN(D5,1)+MIN(E5,1)+MIN(J5,5)+MIN(K5,1)+MIN(L5,1))/18)</f>
         <v/>
       </c>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="9" t="n"/>
       <c r="J5" s="9" t="n"/>
       <c r="K5" s="9" t="n"/>
+      <c r="L5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -1181,13 +1213,14 @@
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="12">
-        <f>IF(A6="","",(MIN(B6,5)+MIN(C6,4)+MIN(D6,1)+MIN(E6,1)+MIN(J6,5)+MIN(K6,1))/17)</f>
+        <f>IF(A6="","",(MIN(B6,5)+MIN(C6,4)+MIN(D6,1)+MIN(E6,1)+MIN(J6,5)+MIN(K6,1)+MIN(L6,1))/18)</f>
         <v/>
       </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
       <c r="J6" s="9" t="n"/>
       <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -1197,13 +1230,14 @@
       <c r="E7" s="9" t="n"/>
       <c r="F7" s="9" t="n"/>
       <c r="G7" s="12">
-        <f>IF(A7="","",(MIN(B7,5)+MIN(C7,4)+MIN(D7,1)+MIN(E7,1)+MIN(J7,5)+MIN(K7,1))/17)</f>
+        <f>IF(A7="","",(MIN(B7,5)+MIN(C7,4)+MIN(D7,1)+MIN(E7,1)+MIN(J7,5)+MIN(K7,1)+MIN(L7,1))/18)</f>
         <v/>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
       <c r="J7" s="9" t="n"/>
       <c r="K7" s="9" t="n"/>
+      <c r="L7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -1213,13 +1247,14 @@
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="9" t="n"/>
       <c r="G8" s="12">
-        <f>IF(A8="","",(MIN(B8,5)+MIN(C8,4)+MIN(D8,1)+MIN(E8,1)+MIN(J8,5)+MIN(K8,1))/17)</f>
+        <f>IF(A8="","",(MIN(B8,5)+MIN(C8,4)+MIN(D8,1)+MIN(E8,1)+MIN(J8,5)+MIN(K8,1)+MIN(L8,1))/18)</f>
         <v/>
       </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -1229,13 +1264,14 @@
       <c r="E9" s="9" t="n"/>
       <c r="F9" s="9" t="n"/>
       <c r="G9" s="12">
-        <f>IF(A9="","",(MIN(B9,5)+MIN(C9,4)+MIN(D9,1)+MIN(E9,1)+MIN(J9,5)+MIN(K9,1))/17)</f>
+        <f>IF(A9="","",(MIN(B9,5)+MIN(C9,4)+MIN(D9,1)+MIN(E9,1)+MIN(J9,5)+MIN(K9,1)+MIN(L9,1))/18)</f>
         <v/>
       </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
       <c r="J9" s="9" t="n"/>
       <c r="K9" s="9" t="n"/>
+      <c r="L9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -1245,13 +1281,14 @@
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
       <c r="G10" s="12">
-        <f>IF(A10="","",(MIN(B10,5)+MIN(C10,4)+MIN(D10,1)+MIN(E10,1)+MIN(J10,5)+MIN(K10,1))/17)</f>
+        <f>IF(A10="","",(MIN(B10,5)+MIN(C10,4)+MIN(D10,1)+MIN(E10,1)+MIN(J10,5)+MIN(K10,1)+MIN(L10,1))/18)</f>
         <v/>
       </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="9" t="n"/>
+      <c r="L10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -1261,13 +1298,14 @@
       <c r="E11" s="9" t="n"/>
       <c r="F11" s="9" t="n"/>
       <c r="G11" s="12">
-        <f>IF(A11="","",(MIN(B11,5)+MIN(C11,4)+MIN(D11,1)+MIN(E11,1)+MIN(J11,5)+MIN(K11,1))/17)</f>
+        <f>IF(A11="","",(MIN(B11,5)+MIN(C11,4)+MIN(D11,1)+MIN(E11,1)+MIN(J11,5)+MIN(K11,1)+MIN(L11,1))/18)</f>
         <v/>
       </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -1277,13 +1315,14 @@
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="9" t="n"/>
       <c r="G12" s="12">
-        <f>IF(A12="","",(MIN(B12,5)+MIN(C12,4)+MIN(D12,1)+MIN(E12,1)+MIN(J12,5)+MIN(K12,1))/17)</f>
+        <f>IF(A12="","",(MIN(B12,5)+MIN(C12,4)+MIN(D12,1)+MIN(E12,1)+MIN(J12,5)+MIN(K12,1)+MIN(L12,1))/18)</f>
         <v/>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -1293,13 +1332,14 @@
       <c r="E13" s="9" t="n"/>
       <c r="F13" s="9" t="n"/>
       <c r="G13" s="12">
-        <f>IF(A13="","",(MIN(B13,5)+MIN(C13,4)+MIN(D13,1)+MIN(E13,1)+MIN(J13,5)+MIN(K13,1))/17)</f>
+        <f>IF(A13="","",(MIN(B13,5)+MIN(C13,4)+MIN(D13,1)+MIN(E13,1)+MIN(J13,5)+MIN(K13,1)+MIN(L13,1))/18)</f>
         <v/>
       </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="n"/>
+      <c r="L13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -1309,13 +1349,14 @@
       <c r="E14" s="9" t="n"/>
       <c r="F14" s="9" t="n"/>
       <c r="G14" s="12">
-        <f>IF(A14="","",(MIN(B14,5)+MIN(C14,4)+MIN(D14,1)+MIN(E14,1)+MIN(J14,5)+MIN(K14,1))/17)</f>
+        <f>IF(A14="","",(MIN(B14,5)+MIN(C14,4)+MIN(D14,1)+MIN(E14,1)+MIN(J14,5)+MIN(K14,1)+MIN(L14,1))/18)</f>
         <v/>
       </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
       <c r="J14" s="9" t="n"/>
       <c r="K14" s="9" t="n"/>
+      <c r="L14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -1325,13 +1366,14 @@
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="9" t="n"/>
       <c r="G15" s="12">
-        <f>IF(A15="","",(MIN(B15,5)+MIN(C15,4)+MIN(D15,1)+MIN(E15,1)+MIN(J15,5)+MIN(K15,1))/17)</f>
+        <f>IF(A15="","",(MIN(B15,5)+MIN(C15,4)+MIN(D15,1)+MIN(E15,1)+MIN(J15,5)+MIN(K15,1)+MIN(L15,1))/18)</f>
         <v/>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
+      <c r="L15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -1341,13 +1383,14 @@
       <c r="E16" s="9" t="n"/>
       <c r="F16" s="9" t="n"/>
       <c r="G16" s="12">
-        <f>IF(A16="","",(MIN(B16,5)+MIN(C16,4)+MIN(D16,1)+MIN(E16,1)+MIN(J16,5)+MIN(K16,1))/17)</f>
+        <f>IF(A16="","",(MIN(B16,5)+MIN(C16,4)+MIN(D16,1)+MIN(E16,1)+MIN(J16,5)+MIN(K16,1)+MIN(L16,1))/18)</f>
         <v/>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
       <c r="J16" s="9" t="n"/>
       <c r="K16" s="9" t="n"/>
+      <c r="L16" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -3025,7 +3068,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Reel,Carrossel,Newsletter,Short,Live YouTube"</formula1>
+      <formula1>"Reel,Carrossel,Newsletter,Short,Live YouTube,Vídeo YouTube"</formula1>
     </dataValidation>
     <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Gabriel,Liliane,Outro"</formula1>
@@ -3044,7 +3087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3061,10 +3104,11 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
     <col width="34" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3147,20 +3191,25 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
+          <t>YouTube: CTR da thumb %</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
           <t>YouTube: cliques no link da newsletter</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>O que funcionou</t>
         </is>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>O que não funcionou</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>O que vou testar na semana que vem</t>
         </is>
@@ -3185,9 +3234,10 @@
       <c r="M4" s="9" t="n"/>
       <c r="N4" s="9" t="n"/>
       <c r="O4" s="9" t="n"/>
-      <c r="P4" s="17" t="n"/>
+      <c r="P4" s="9" t="n"/>
       <c r="Q4" s="17" t="n"/>
       <c r="R4" s="17" t="n"/>
+      <c r="S4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -3208,9 +3258,10 @@
       <c r="M5" s="9" t="n"/>
       <c r="N5" s="9" t="n"/>
       <c r="O5" s="9" t="n"/>
-      <c r="P5" s="17" t="n"/>
+      <c r="P5" s="9" t="n"/>
       <c r="Q5" s="17" t="n"/>
       <c r="R5" s="17" t="n"/>
+      <c r="S5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -3231,9 +3282,10 @@
       <c r="M6" s="9" t="n"/>
       <c r="N6" s="9" t="n"/>
       <c r="O6" s="9" t="n"/>
-      <c r="P6" s="17" t="n"/>
+      <c r="P6" s="9" t="n"/>
       <c r="Q6" s="17" t="n"/>
       <c r="R6" s="17" t="n"/>
+      <c r="S6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -3254,9 +3306,10 @@
       <c r="M7" s="9" t="n"/>
       <c r="N7" s="9" t="n"/>
       <c r="O7" s="9" t="n"/>
-      <c r="P7" s="17" t="n"/>
+      <c r="P7" s="9" t="n"/>
       <c r="Q7" s="17" t="n"/>
       <c r="R7" s="17" t="n"/>
+      <c r="S7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -3277,9 +3330,10 @@
       <c r="M8" s="9" t="n"/>
       <c r="N8" s="9" t="n"/>
       <c r="O8" s="9" t="n"/>
-      <c r="P8" s="17" t="n"/>
+      <c r="P8" s="9" t="n"/>
       <c r="Q8" s="17" t="n"/>
       <c r="R8" s="17" t="n"/>
+      <c r="S8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -3300,9 +3354,10 @@
       <c r="M9" s="9" t="n"/>
       <c r="N9" s="9" t="n"/>
       <c r="O9" s="9" t="n"/>
-      <c r="P9" s="17" t="n"/>
+      <c r="P9" s="9" t="n"/>
       <c r="Q9" s="17" t="n"/>
       <c r="R9" s="17" t="n"/>
+      <c r="S9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -3323,9 +3378,10 @@
       <c r="M10" s="9" t="n"/>
       <c r="N10" s="9" t="n"/>
       <c r="O10" s="9" t="n"/>
-      <c r="P10" s="17" t="n"/>
+      <c r="P10" s="9" t="n"/>
       <c r="Q10" s="17" t="n"/>
       <c r="R10" s="17" t="n"/>
+      <c r="S10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -3346,9 +3402,10 @@
       <c r="M11" s="9" t="n"/>
       <c r="N11" s="9" t="n"/>
       <c r="O11" s="9" t="n"/>
-      <c r="P11" s="17" t="n"/>
+      <c r="P11" s="9" t="n"/>
       <c r="Q11" s="17" t="n"/>
       <c r="R11" s="17" t="n"/>
+      <c r="S11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -3369,9 +3426,10 @@
       <c r="M12" s="9" t="n"/>
       <c r="N12" s="9" t="n"/>
       <c r="O12" s="9" t="n"/>
-      <c r="P12" s="17" t="n"/>
+      <c r="P12" s="9" t="n"/>
       <c r="Q12" s="17" t="n"/>
       <c r="R12" s="17" t="n"/>
+      <c r="S12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -3392,9 +3450,10 @@
       <c r="M13" s="9" t="n"/>
       <c r="N13" s="9" t="n"/>
       <c r="O13" s="9" t="n"/>
-      <c r="P13" s="17" t="n"/>
+      <c r="P13" s="9" t="n"/>
       <c r="Q13" s="17" t="n"/>
       <c r="R13" s="17" t="n"/>
+      <c r="S13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -3415,9 +3474,10 @@
       <c r="M14" s="9" t="n"/>
       <c r="N14" s="9" t="n"/>
       <c r="O14" s="9" t="n"/>
-      <c r="P14" s="17" t="n"/>
+      <c r="P14" s="9" t="n"/>
       <c r="Q14" s="17" t="n"/>
       <c r="R14" s="17" t="n"/>
+      <c r="S14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -3438,9 +3498,10 @@
       <c r="M15" s="9" t="n"/>
       <c r="N15" s="9" t="n"/>
       <c r="O15" s="9" t="n"/>
-      <c r="P15" s="17" t="n"/>
+      <c r="P15" s="9" t="n"/>
       <c r="Q15" s="17" t="n"/>
       <c r="R15" s="17" t="n"/>
+      <c r="S15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -3461,9 +3522,10 @@
       <c r="M16" s="9" t="n"/>
       <c r="N16" s="9" t="n"/>
       <c r="O16" s="9" t="n"/>
-      <c r="P16" s="17" t="n"/>
+      <c r="P16" s="9" t="n"/>
       <c r="Q16" s="17" t="n"/>
       <c r="R16" s="17" t="n"/>
+      <c r="S16" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3490,7 +3552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3704,7 +3766,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>YOUTUBE (live): título com a palavra que a pessoa buscaria, capa com foto real e texto grande, descrição com resumo, momentos principais e link da newsletter, comentário fixado com o link.</t>
+          <t>YOUTUBE (thumb): tem rosto grande com expressão forte, até 4 palavras, flecha ou círculo no elemento principal, e dá para ler no celular. Nunca só nome ou texto.</t>
         </is>
       </c>
     </row>
@@ -3715,6 +3777,30 @@
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>YOUTUBE (vídeo roteirizado): a promessa do vídeo aparece nos primeiros 30 segundos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>YOUTUBE (live): título com a palavra que a pessoa buscaria, capa com foto real e texto grande, descrição com resumo, momentos principais e link da newsletter, comentário fixado com o link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>CAMPANHA: se fala de oferta, diz exatamente o que a página de destino diz (mesma frase, número, prazo).</t>
         </is>

</xml_diff>

<commit_message>
Plano de conteúdo: venda como objetivo final, ritmo de venda, produto da semana e stories
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. KPIs da semana" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Checklist do roteiro" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Calendário de captura" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Produto da semana" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -503,361 +504,445 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AS CAMADAS (ler primeiro)</t>
+          <t>OBJETIVO FINAL (ler primeiro)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>O PRINCIPAL DA SEMANA é transformar seguidor em base (e-mail). O número que mais importa: e-mails novos + cliques na newsletter.</t>
+          <t>VENDA. Tudo existe para vender mais: alcance e engajamento trazem gente nova; a base aquecida (seguidores que confiam + e-mail) é quem compra. Venda ← base aquecida ← alcance e engajamento.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CAMADA 1 · O CENTRO</t>
+          <t>AS CAMADAS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Tema da semana (vem da live) → NEWSLETTER. É o produto da semana e o que mantém a base quente.</t>
+          <t>No dia a dia, o trabalho principal é transformar seguidor em base (e-mail) e aquecer essa base. Mas toda semana também tem venda (ver RITMO DE VENDA).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>CAMADA 1 · O CENTRO</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Tema da semana (vem da live) → NEWSLETTER. É o produto da semana e o que mantém a base quente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>CAMADA 2 · A PONTE</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Criativo de captura ("comenta e recebe"). Leva a pessoa do Instagram para dentro da base.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>CAMADA 3 · O COMBUSTÍVEL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Reels, carrosséis e YouTube. Atraem gente nova e aquecem quem já segue. Uns 3 por semana no tema da semana; o resto nos assuntos fixos ligados às formações (para o perfil não ficar repetitivo).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>CARROSSEL DA NEWSLETTER</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>NUNCA abrir com "o tema da newsletter desta semana". A capa é a ideia mais surpreendente que está DENTRO da newsletter, algo que quebra a cabeça e faz rolar. Só no último slide a pessoa descobre que aquilo é um pedaço da newsletter: "Isso saiu na nossa newsletter desta semana. Quer receber as próximas? Comenta NEWS."</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>COMO SOMOS MEDIDOS (3 níveis)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>1) TODA SEMANA, ENTREGAS (aba 3): fiz o que combinei? Meta 100%. 2) TODA SEMANA, KPIs (aba 5): os números que mostram se a operação está saudável (seguidores novos, engajados, e-mails novos, cliques). Eu trago e comparo com a semana anterior. 3) TODO MÊS, OKR (aba 2): a meta de RESULTADO do mês. É o que diz se o trabalho trouxe resultado. E em cada peça, o PLACAR (aba 4): gancho, retenção e conversão de cada reel e carrossel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>OKR x KPI</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>OKR é o que queremos MUDAR no mês (crescer a base, aumentar cliques). KPI é o que não podemos deixar PIORAR toda semana. OKR muda a cada mês; KPI é sempre o mesmo painel.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>VISÃO</t>
+          <t>OKR x KPI</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t>OKR é o que queremos MUDAR no mês (crescer a base, aumentar cliques). KPI é o que não podemos deixar PIORAR toda semana. OKR muda a cada mês; KPI é sempre o mesmo painel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>RESPONSÁVEL</t>
+          <t>RITMO DE VENDA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t>Toda semana tem venda. Feed: das 9 peças, 2 são de venda (caso real, depoimento, "isso a gente ensina na formação X"), umas 7 são conteúdo. Stories: todo dia pelo menos 1 story de venda, com link. Newsletter: sempre com o bloco da formação ligada ao tema. YouTube: link da formação na descrição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>QUEM APARECE</t>
+          <t>PRODUTO DA SEMANA</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+          <t>Depois da Black, a FSA vende tudo o que tem, sem oferta: 2 pós, 7 cursos e a mentoria. Cada semana tem UM produto em destaque, ligado ao tema da live (live de exames → formação de exames). É esse produto que aparece nas 2 peças de venda, no story de venda e no bloco da newsletter. Calendário na aba 8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>O CENTRO DA SEMANA</t>
+          <t>DEPOIS DA BLACK (01/11 em diante)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
+          <t>As 2 primeiras semanas de novembro são só conteúdo, sem venda: a base acabou de receber muita oferta. A venda contínua começa na 3ª semana. Nada de desconto nem "última chance": preço cheio, valor explicado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ENTREGAS DA SEMANA</t>
+          <t>MENTORIA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter + YouTube (5 Shorts + 1 vídeo roteirizado + a live da semana). Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>É venda de alto valor: não vai para link de compra direto. A chamada leva para conversa (aplicação ou WhatsApp). Entra como produto da semana 1 vez por mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>YOUTUBE: SHORTS</t>
+          <t>STORIES (todo dia)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Os 5 reels da semana sobem também como Shorts no YouTube. Sem roteiro novo: é repostar, com título próprio para o YouTube.</t>
+          <t>Ela planeja e roteiriza os stories da semana; quem aparece grava. Sequência diária de 5 a 8 stories: 1) bastidor ou rotina (gente real); 2) conteúdo rápido; 3) interação (enquete, caixinha, quiz); 4) prova (depoimento, print autorizado); 5) venda do produto da semana, com link.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>YOUTUBE: A LIVE DA SEMANA</t>
+          <t>LINKS COM RASTREIO</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>A gravação da live sobe no YouTube toda semana. O trabalho dela: título forte (com a palavra que a pessoa buscaria no Google), capa com foto real e texto grande, descrição com o resumo, os momentos principais e o link da newsletter. Tempo: uns 30 minutos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
+          <t>Cada canal tem link próprio com rastreio (UTM): bio, stories, newsletter, YouTube. Assim a Hotmart mostra de onde veio cada venda. A pessoa das automações monta. Sem isso, não dá para saber qual conteúdo vendeu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>YOUTUBE: VÍDEO ROTEIRIZADO</t>
+          <t>VISÃO</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>1 por semana, de 8 a 15 minutos, gravado pelo Gabriel ou pela Liliane. Usa o MESMO tema da newsletter da semana, mais aprofundado: a pesquisa já está feita, então o trabalho é o roteiro. Estrutura: gancho nos primeiros 30 segundos (a promessa do vídeo), desenvolvimento em blocos, caso prático, chamada para a newsletter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="75" customHeight="1">
+          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>YOUTUBE: THUMB (CAPA)</t>
+          <t>RESPONSÁVEL</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Toda thumb tem ROSTO, nunca só nome ou texto. Rosto grande, com expressão que chama atenção (surpresa, dúvida, preocupação, apontando). Foto real do professor, feita para a thumb. Até 4 palavras em letra grande, que completam o título sem repetir. Flecha ou círculo apontando para o elemento principal (o exame, o alimento, o número). Contraste forte. Testar se dá para ler no tamanho de celular.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
+          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>YOUTUBE: O PAPEL</t>
+          <t>QUEM APARECE</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. O número que mostra se a thumb funciona é a TAXA DE CLIQUES (CTR) das impressões, no YouTube Studio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
+          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+          <t>O CENTRO DA SEMANA</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+          <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>MATERIAL DE CAPTURA</t>
+          <t>ENTREGAS DA SEMANA</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+          <t>5 roteiros de reels + 4 carrosséis + 1 newsletter + YouTube (5 Shorts + 1 vídeo roteirizado + a live da semana). Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ROTINA (D = dia da live)</t>
+          <t>YOUTUBE: SHORTS</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
+          <t>Os 5 reels da semana sobem também como Shorts no YouTube. Sem roteiro novo: é repostar, com título próprio para o YouTube.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>YOUTUBE: A LIVE DA SEMANA</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>A gravação da live sobe no YouTube toda semana. O trabalho dela: título forte (com a palavra que a pessoa buscaria no Google), capa com foto real e texto grande, descrição com o resumo, os momentos principais e o link da newsletter. Tempo: uns 30 minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>YOUTUBE: VÍDEO ROTEIRIZADO</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>1 por semana, de 8 a 15 minutos, gravado pelo Gabriel ou pela Liliane. Usa o MESMO tema da newsletter da semana, mais aprofundado: a pesquisa já está feita, então o trabalho é o roteiro. Estrutura: gancho nos primeiros 30 segundos (a promessa do vídeo), desenvolvimento em blocos, caso prático, chamada para a newsletter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="75" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>YOUTUBE: THUMB (CAPA)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Toda thumb tem ROSTO, nunca só nome ou texto. Rosto grande, com expressão que chama atenção (surpresa, dúvida, preocupação, apontando). Foto real do professor, feita para a thumb. Até 4 palavras em letra grande, que completam o título sem repetir. Flecha ou círculo apontando para o elemento principal (o exame, o alimento, o número). Contraste forte. Testar se dá para ler no tamanho de celular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>YOUTUBE: O PAPEL</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. O número que mostra se a thumb funciona é a TAXA DE CLIQUES (CTR) das impressões, no YouTube Studio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>MATERIAL DE CAPTURA</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ROTINA (D = dia da live)</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>IMAGENS (responsabilidade dela)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Todo roteiro e carrossel sai com as imagens escolhidas, não só o texto. Imagem REAL, nunca de IA: professores, aulas, bastidores, prova (depoimentos e prints de alunos), e imagem daquilo que se está falando (o exame, o suplemento, o alimento). Muita imagem.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>BANCO DE IMAGENS</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>ARTE DO CARROSSEL</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>AUTORIZAÇÃO DE IMAGEM</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>APROVAÇÃO</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>PRIORIDADE SE O TEMPO APERTAR</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>1) Newsletter  2) Criativo de captura  3) Vídeo roteirizado do YouTube  4) Carrosséis  5) Reels  6) Live no YouTube  7) Shorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>1) Stories do dia (com o de venda)  2) Newsletter  3) As 2 peças de venda  4) Criativo de captura  5) Vídeo roteirizado do YouTube  6) Carrosséis e reels  7) Live e Shorts no YouTube</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>A META É RESULTADO</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>TODA SEMANA, 3 LINHAS</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>O que funcionou. O que não funcionou. O que vou testar na semana que vem. (aba 5)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="45" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>REGRAS QUE NÃO MUDAM</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>BASE DE E-MAIL</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Reaquecer em ordem: semanas 1 e 2 só para quem abriu ou clicou nos últimos 6 meses; semana 3 campanha de reativação para os parados; depois tirar do envio quem não abre há 12 meses. Spam acima de 0,1%: parar e corrigir.</t>
         </is>
@@ -874,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -909,7 +994,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta.</t>
+          <t>Vender mais com o conteúdo: crescer a audiência, aquecer a base e converter em vendas dos nossos produtos.</t>
         </is>
       </c>
     </row>
@@ -953,12 +1038,12 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>KR1. Gancho e retenção dos reels</t>
+          <t>KR1. Vendas vindas do conteúdo</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>% dos reels do mês com retenção (tempo médio ÷ duração) acima da linha de base</t>
+          <t>Vendas no mês com origem em bio, stories, newsletter e YouTube (links com rastreio na Hotmart)</t>
         </is>
       </c>
       <c r="C6" s="9" t="n"/>
@@ -973,12 +1058,12 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>KR2. Base nova vinda do Instagram</t>
+          <t>KR2. Seguidores novos</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>E-mails novos gerados pelos criativos de captura no mês</t>
+          <t>Seguidores novos no mês (Instagram + inscritos no YouTube)</t>
         </is>
       </c>
       <c r="C7" s="9" t="n"/>
@@ -993,12 +1078,12 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>KR3. Engajamento que importa</t>
+          <t>KR3. Gancho e retenção dos reels</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>(Comentários + salvamentos + compartilhamentos) ÷ alcance, média do mês</t>
+          <t>% dos reels do mês com retenção (tempo médio ÷ duração) acima da linha de base</t>
         </is>
       </c>
       <c r="C8" s="9" t="n"/>
@@ -1013,12 +1098,12 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>KR4. Newsletter viva</t>
+          <t>KR4. Base nova vinda do Instagram</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Taxa média de cliques das newsletters do mês</t>
+          <t>E-mails novos gerados pelos criativos de captura no mês</t>
         </is>
       </c>
       <c r="C9" s="9" t="n"/>
@@ -1033,12 +1118,12 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>KR5. Base reativada</t>
+          <t>KR5. Engajamento que importa</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Contatos parados que voltaram a abrir ou clicar no mês</t>
+          <t>(Comentários + salvamentos + compartilhamentos) ÷ alcance, média do mês</t>
         </is>
       </c>
       <c r="C10" s="9" t="n"/>
@@ -1050,25 +1135,65 @@
       </c>
       <c r="G10" s="11" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Indicador de apoio (não é meta):</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Seguidores novos no mês. Acompanhar, mas não perseguir: meta de seguidor puxa conteúdo que viraliza e não vende.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>KR6. Newsletter viva</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Taxa média de cliques das newsletters do mês</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="10">
+        <f>IFERROR(E11/D11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>KR7. Base reativada</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Contatos parados que voltaram a abrir ou clicar no mês</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="10">
+        <f>IFERROR(E12/D12,"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Atenção:</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Seguidor é meta, mas sempre junto com engajamento e venda. Seguidor que vem de conteúdo viral sem relação com a FSA não compra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Regra:</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>No 1º mês, as duas primeiras semanas viram a linha de base. A partir do 2º mês, a meta é superar a linha de base do mês anterior. Bater 70% do OKR já é bom resultado.</t>
         </is>
@@ -1085,7 +1210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1100,6 +1225,8 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1168,6 +1295,16 @@
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Vídeo roteirizado no YouTube (1)</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>Dias com stories planejados (meta 7)</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Peças de venda no feed (meta 2)</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1316,7 @@
       <c r="E4" s="9" t="n"/>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="12">
-        <f>IF(A4="","",(MIN(B4,5)+MIN(C4,4)+MIN(D4,1)+MIN(E4,1)+MIN(J4,5)+MIN(K4,1)+MIN(L4,1))/18)</f>
+        <f>IF(A4="","",(MIN(B4,5)+MIN(C4,4)+MIN(D4,1)+MIN(E4,1)+MIN(J4,5)+MIN(K4,1)+MIN(L4,1)+MIN(M4,7)+MIN(N4,2))/27)</f>
         <v/>
       </c>
       <c r="H4" s="9" t="n"/>
@@ -1187,6 +1324,8 @@
       <c r="J4" s="9" t="n"/>
       <c r="K4" s="9" t="n"/>
       <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="n"/>
+      <c r="N4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -1196,7 +1335,7 @@
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="9" t="n"/>
       <c r="G5" s="12">
-        <f>IF(A5="","",(MIN(B5,5)+MIN(C5,4)+MIN(D5,1)+MIN(E5,1)+MIN(J5,5)+MIN(K5,1)+MIN(L5,1))/18)</f>
+        <f>IF(A5="","",(MIN(B5,5)+MIN(C5,4)+MIN(D5,1)+MIN(E5,1)+MIN(J5,5)+MIN(K5,1)+MIN(L5,1)+MIN(M5,7)+MIN(N5,2))/27)</f>
         <v/>
       </c>
       <c r="H5" s="9" t="n"/>
@@ -1204,6 +1343,8 @@
       <c r="J5" s="9" t="n"/>
       <c r="K5" s="9" t="n"/>
       <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -1213,7 +1354,7 @@
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="12">
-        <f>IF(A6="","",(MIN(B6,5)+MIN(C6,4)+MIN(D6,1)+MIN(E6,1)+MIN(J6,5)+MIN(K6,1)+MIN(L6,1))/18)</f>
+        <f>IF(A6="","",(MIN(B6,5)+MIN(C6,4)+MIN(D6,1)+MIN(E6,1)+MIN(J6,5)+MIN(K6,1)+MIN(L6,1)+MIN(M6,7)+MIN(N6,2))/27)</f>
         <v/>
       </c>
       <c r="H6" s="9" t="n"/>
@@ -1221,6 +1362,8 @@
       <c r="J6" s="9" t="n"/>
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -1230,7 +1373,7 @@
       <c r="E7" s="9" t="n"/>
       <c r="F7" s="9" t="n"/>
       <c r="G7" s="12">
-        <f>IF(A7="","",(MIN(B7,5)+MIN(C7,4)+MIN(D7,1)+MIN(E7,1)+MIN(J7,5)+MIN(K7,1)+MIN(L7,1))/18)</f>
+        <f>IF(A7="","",(MIN(B7,5)+MIN(C7,4)+MIN(D7,1)+MIN(E7,1)+MIN(J7,5)+MIN(K7,1)+MIN(L7,1)+MIN(M7,7)+MIN(N7,2))/27)</f>
         <v/>
       </c>
       <c r="H7" s="9" t="n"/>
@@ -1238,6 +1381,8 @@
       <c r="J7" s="9" t="n"/>
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
+      <c r="M7" s="9" t="n"/>
+      <c r="N7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -1247,7 +1392,7 @@
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="9" t="n"/>
       <c r="G8" s="12">
-        <f>IF(A8="","",(MIN(B8,5)+MIN(C8,4)+MIN(D8,1)+MIN(E8,1)+MIN(J8,5)+MIN(K8,1)+MIN(L8,1))/18)</f>
+        <f>IF(A8="","",(MIN(B8,5)+MIN(C8,4)+MIN(D8,1)+MIN(E8,1)+MIN(J8,5)+MIN(K8,1)+MIN(L8,1)+MIN(M8,7)+MIN(N8,2))/27)</f>
         <v/>
       </c>
       <c r="H8" s="9" t="n"/>
@@ -1255,6 +1400,8 @@
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -1264,7 +1411,7 @@
       <c r="E9" s="9" t="n"/>
       <c r="F9" s="9" t="n"/>
       <c r="G9" s="12">
-        <f>IF(A9="","",(MIN(B9,5)+MIN(C9,4)+MIN(D9,1)+MIN(E9,1)+MIN(J9,5)+MIN(K9,1)+MIN(L9,1))/18)</f>
+        <f>IF(A9="","",(MIN(B9,5)+MIN(C9,4)+MIN(D9,1)+MIN(E9,1)+MIN(J9,5)+MIN(K9,1)+MIN(L9,1)+MIN(M9,7)+MIN(N9,2))/27)</f>
         <v/>
       </c>
       <c r="H9" s="9" t="n"/>
@@ -1272,6 +1419,8 @@
       <c r="J9" s="9" t="n"/>
       <c r="K9" s="9" t="n"/>
       <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -1281,7 +1430,7 @@
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
       <c r="G10" s="12">
-        <f>IF(A10="","",(MIN(B10,5)+MIN(C10,4)+MIN(D10,1)+MIN(E10,1)+MIN(J10,5)+MIN(K10,1)+MIN(L10,1))/18)</f>
+        <f>IF(A10="","",(MIN(B10,5)+MIN(C10,4)+MIN(D10,1)+MIN(E10,1)+MIN(J10,5)+MIN(K10,1)+MIN(L10,1)+MIN(M10,7)+MIN(N10,2))/27)</f>
         <v/>
       </c>
       <c r="H10" s="9" t="n"/>
@@ -1289,6 +1438,8 @@
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -1298,7 +1449,7 @@
       <c r="E11" s="9" t="n"/>
       <c r="F11" s="9" t="n"/>
       <c r="G11" s="12">
-        <f>IF(A11="","",(MIN(B11,5)+MIN(C11,4)+MIN(D11,1)+MIN(E11,1)+MIN(J11,5)+MIN(K11,1)+MIN(L11,1))/18)</f>
+        <f>IF(A11="","",(MIN(B11,5)+MIN(C11,4)+MIN(D11,1)+MIN(E11,1)+MIN(J11,5)+MIN(K11,1)+MIN(L11,1)+MIN(M11,7)+MIN(N11,2))/27)</f>
         <v/>
       </c>
       <c r="H11" s="9" t="n"/>
@@ -1306,6 +1457,8 @@
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="9" t="n"/>
       <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -1315,7 +1468,7 @@
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="9" t="n"/>
       <c r="G12" s="12">
-        <f>IF(A12="","",(MIN(B12,5)+MIN(C12,4)+MIN(D12,1)+MIN(E12,1)+MIN(J12,5)+MIN(K12,1)+MIN(L12,1))/18)</f>
+        <f>IF(A12="","",(MIN(B12,5)+MIN(C12,4)+MIN(D12,1)+MIN(E12,1)+MIN(J12,5)+MIN(K12,1)+MIN(L12,1)+MIN(M12,7)+MIN(N12,2))/27)</f>
         <v/>
       </c>
       <c r="H12" s="9" t="n"/>
@@ -1323,6 +1476,8 @@
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -1332,7 +1487,7 @@
       <c r="E13" s="9" t="n"/>
       <c r="F13" s="9" t="n"/>
       <c r="G13" s="12">
-        <f>IF(A13="","",(MIN(B13,5)+MIN(C13,4)+MIN(D13,1)+MIN(E13,1)+MIN(J13,5)+MIN(K13,1)+MIN(L13,1))/18)</f>
+        <f>IF(A13="","",(MIN(B13,5)+MIN(C13,4)+MIN(D13,1)+MIN(E13,1)+MIN(J13,5)+MIN(K13,1)+MIN(L13,1)+MIN(M13,7)+MIN(N13,2))/27)</f>
         <v/>
       </c>
       <c r="H13" s="9" t="n"/>
@@ -1340,6 +1495,8 @@
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="n"/>
       <c r="L13" s="9" t="n"/>
+      <c r="M13" s="9" t="n"/>
+      <c r="N13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -1349,7 +1506,7 @@
       <c r="E14" s="9" t="n"/>
       <c r="F14" s="9" t="n"/>
       <c r="G14" s="12">
-        <f>IF(A14="","",(MIN(B14,5)+MIN(C14,4)+MIN(D14,1)+MIN(E14,1)+MIN(J14,5)+MIN(K14,1)+MIN(L14,1))/18)</f>
+        <f>IF(A14="","",(MIN(B14,5)+MIN(C14,4)+MIN(D14,1)+MIN(E14,1)+MIN(J14,5)+MIN(K14,1)+MIN(L14,1)+MIN(M14,7)+MIN(N14,2))/27)</f>
         <v/>
       </c>
       <c r="H14" s="9" t="n"/>
@@ -1357,6 +1514,8 @@
       <c r="J14" s="9" t="n"/>
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
+      <c r="M14" s="9" t="n"/>
+      <c r="N14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -1366,7 +1525,7 @@
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="9" t="n"/>
       <c r="G15" s="12">
-        <f>IF(A15="","",(MIN(B15,5)+MIN(C15,4)+MIN(D15,1)+MIN(E15,1)+MIN(J15,5)+MIN(K15,1)+MIN(L15,1))/18)</f>
+        <f>IF(A15="","",(MIN(B15,5)+MIN(C15,4)+MIN(D15,1)+MIN(E15,1)+MIN(J15,5)+MIN(K15,1)+MIN(L15,1)+MIN(M15,7)+MIN(N15,2))/27)</f>
         <v/>
       </c>
       <c r="H15" s="9" t="n"/>
@@ -1374,6 +1533,8 @@
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
       <c r="L15" s="9" t="n"/>
+      <c r="M15" s="9" t="n"/>
+      <c r="N15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -1383,7 +1544,7 @@
       <c r="E16" s="9" t="n"/>
       <c r="F16" s="9" t="n"/>
       <c r="G16" s="12">
-        <f>IF(A16="","",(MIN(B16,5)+MIN(C16,4)+MIN(D16,1)+MIN(E16,1)+MIN(J16,5)+MIN(K16,1)+MIN(L16,1))/18)</f>
+        <f>IF(A16="","",(MIN(B16,5)+MIN(C16,4)+MIN(D16,1)+MIN(E16,1)+MIN(J16,5)+MIN(K16,1)+MIN(L16,1)+MIN(M16,7)+MIN(N16,2))/27)</f>
         <v/>
       </c>
       <c r="H16" s="9" t="n"/>
@@ -1391,6 +1552,8 @@
       <c r="J16" s="9" t="n"/>
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
+      <c r="M16" s="9" t="n"/>
+      <c r="N16" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -3068,7 +3231,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Reel,Carrossel,Newsletter,Short,Live YouTube,Vídeo YouTube"</formula1>
+      <formula1>"Reel,Carrossel,Newsletter,Short,Live YouTube,Vídeo YouTube,Venda (feed)"</formula1>
     </dataValidation>
     <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Gabriel,Liliane,Outro"</formula1>
@@ -3087,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3106,9 +3269,16 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="34" customWidth="1" min="18" max="18"/>
-    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="34" customWidth="1" min="24" max="24"/>
+    <col width="34" customWidth="1" min="25" max="25"/>
+    <col width="34" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3201,15 +3371,50 @@
       </c>
       <c r="Q3" s="6" t="inlineStr">
         <is>
+          <t>Stories: visualizações médias</t>
+        </is>
+      </c>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>Stories: respostas (enquete/caixinha)</t>
+        </is>
+      </c>
+      <c r="S3" s="6" t="inlineStr">
+        <is>
+          <t>Stories: cliques no link</t>
+        </is>
+      </c>
+      <c r="T3" s="6" t="inlineStr">
+        <is>
+          <t>Vendas: bio</t>
+        </is>
+      </c>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t>Vendas: stories</t>
+        </is>
+      </c>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>Vendas: newsletter</t>
+        </is>
+      </c>
+      <c r="W3" s="6" t="inlineStr">
+        <is>
+          <t>Vendas: YouTube</t>
+        </is>
+      </c>
+      <c r="X3" s="6" t="inlineStr">
+        <is>
           <t>O que funcionou</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="Y3" s="6" t="inlineStr">
         <is>
           <t>O que não funcionou</t>
         </is>
       </c>
-      <c r="S3" s="6" t="inlineStr">
+      <c r="Z3" s="6" t="inlineStr">
         <is>
           <t>O que vou testar na semana que vem</t>
         </is>
@@ -3235,9 +3440,16 @@
       <c r="N4" s="9" t="n"/>
       <c r="O4" s="9" t="n"/>
       <c r="P4" s="9" t="n"/>
-      <c r="Q4" s="17" t="n"/>
-      <c r="R4" s="17" t="n"/>
-      <c r="S4" s="17" t="n"/>
+      <c r="Q4" s="9" t="n"/>
+      <c r="R4" s="9" t="n"/>
+      <c r="S4" s="9" t="n"/>
+      <c r="T4" s="9" t="n"/>
+      <c r="U4" s="9" t="n"/>
+      <c r="V4" s="9" t="n"/>
+      <c r="W4" s="9" t="n"/>
+      <c r="X4" s="17" t="n"/>
+      <c r="Y4" s="17" t="n"/>
+      <c r="Z4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -3259,9 +3471,16 @@
       <c r="N5" s="9" t="n"/>
       <c r="O5" s="9" t="n"/>
       <c r="P5" s="9" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
-      <c r="S5" s="17" t="n"/>
+      <c r="Q5" s="9" t="n"/>
+      <c r="R5" s="9" t="n"/>
+      <c r="S5" s="9" t="n"/>
+      <c r="T5" s="9" t="n"/>
+      <c r="U5" s="9" t="n"/>
+      <c r="V5" s="9" t="n"/>
+      <c r="W5" s="9" t="n"/>
+      <c r="X5" s="17" t="n"/>
+      <c r="Y5" s="17" t="n"/>
+      <c r="Z5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -3283,9 +3502,16 @@
       <c r="N6" s="9" t="n"/>
       <c r="O6" s="9" t="n"/>
       <c r="P6" s="9" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="17" t="n"/>
-      <c r="S6" s="17" t="n"/>
+      <c r="Q6" s="9" t="n"/>
+      <c r="R6" s="9" t="n"/>
+      <c r="S6" s="9" t="n"/>
+      <c r="T6" s="9" t="n"/>
+      <c r="U6" s="9" t="n"/>
+      <c r="V6" s="9" t="n"/>
+      <c r="W6" s="9" t="n"/>
+      <c r="X6" s="17" t="n"/>
+      <c r="Y6" s="17" t="n"/>
+      <c r="Z6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -3307,9 +3533,16 @@
       <c r="N7" s="9" t="n"/>
       <c r="O7" s="9" t="n"/>
       <c r="P7" s="9" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="17" t="n"/>
-      <c r="S7" s="17" t="n"/>
+      <c r="Q7" s="9" t="n"/>
+      <c r="R7" s="9" t="n"/>
+      <c r="S7" s="9" t="n"/>
+      <c r="T7" s="9" t="n"/>
+      <c r="U7" s="9" t="n"/>
+      <c r="V7" s="9" t="n"/>
+      <c r="W7" s="9" t="n"/>
+      <c r="X7" s="17" t="n"/>
+      <c r="Y7" s="17" t="n"/>
+      <c r="Z7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -3331,9 +3564,16 @@
       <c r="N8" s="9" t="n"/>
       <c r="O8" s="9" t="n"/>
       <c r="P8" s="9" t="n"/>
-      <c r="Q8" s="17" t="n"/>
-      <c r="R8" s="17" t="n"/>
-      <c r="S8" s="17" t="n"/>
+      <c r="Q8" s="9" t="n"/>
+      <c r="R8" s="9" t="n"/>
+      <c r="S8" s="9" t="n"/>
+      <c r="T8" s="9" t="n"/>
+      <c r="U8" s="9" t="n"/>
+      <c r="V8" s="9" t="n"/>
+      <c r="W8" s="9" t="n"/>
+      <c r="X8" s="17" t="n"/>
+      <c r="Y8" s="17" t="n"/>
+      <c r="Z8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -3355,9 +3595,16 @@
       <c r="N9" s="9" t="n"/>
       <c r="O9" s="9" t="n"/>
       <c r="P9" s="9" t="n"/>
-      <c r="Q9" s="17" t="n"/>
-      <c r="R9" s="17" t="n"/>
-      <c r="S9" s="17" t="n"/>
+      <c r="Q9" s="9" t="n"/>
+      <c r="R9" s="9" t="n"/>
+      <c r="S9" s="9" t="n"/>
+      <c r="T9" s="9" t="n"/>
+      <c r="U9" s="9" t="n"/>
+      <c r="V9" s="9" t="n"/>
+      <c r="W9" s="9" t="n"/>
+      <c r="X9" s="17" t="n"/>
+      <c r="Y9" s="17" t="n"/>
+      <c r="Z9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -3379,9 +3626,16 @@
       <c r="N10" s="9" t="n"/>
       <c r="O10" s="9" t="n"/>
       <c r="P10" s="9" t="n"/>
-      <c r="Q10" s="17" t="n"/>
-      <c r="R10" s="17" t="n"/>
-      <c r="S10" s="17" t="n"/>
+      <c r="Q10" s="9" t="n"/>
+      <c r="R10" s="9" t="n"/>
+      <c r="S10" s="9" t="n"/>
+      <c r="T10" s="9" t="n"/>
+      <c r="U10" s="9" t="n"/>
+      <c r="V10" s="9" t="n"/>
+      <c r="W10" s="9" t="n"/>
+      <c r="X10" s="17" t="n"/>
+      <c r="Y10" s="17" t="n"/>
+      <c r="Z10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
@@ -3403,9 +3657,16 @@
       <c r="N11" s="9" t="n"/>
       <c r="O11" s="9" t="n"/>
       <c r="P11" s="9" t="n"/>
-      <c r="Q11" s="17" t="n"/>
-      <c r="R11" s="17" t="n"/>
-      <c r="S11" s="17" t="n"/>
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="9" t="n"/>
+      <c r="S11" s="9" t="n"/>
+      <c r="T11" s="9" t="n"/>
+      <c r="U11" s="9" t="n"/>
+      <c r="V11" s="9" t="n"/>
+      <c r="W11" s="9" t="n"/>
+      <c r="X11" s="17" t="n"/>
+      <c r="Y11" s="17" t="n"/>
+      <c r="Z11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
@@ -3427,9 +3688,16 @@
       <c r="N12" s="9" t="n"/>
       <c r="O12" s="9" t="n"/>
       <c r="P12" s="9" t="n"/>
-      <c r="Q12" s="17" t="n"/>
-      <c r="R12" s="17" t="n"/>
-      <c r="S12" s="17" t="n"/>
+      <c r="Q12" s="9" t="n"/>
+      <c r="R12" s="9" t="n"/>
+      <c r="S12" s="9" t="n"/>
+      <c r="T12" s="9" t="n"/>
+      <c r="U12" s="9" t="n"/>
+      <c r="V12" s="9" t="n"/>
+      <c r="W12" s="9" t="n"/>
+      <c r="X12" s="17" t="n"/>
+      <c r="Y12" s="17" t="n"/>
+      <c r="Z12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
@@ -3451,9 +3719,16 @@
       <c r="N13" s="9" t="n"/>
       <c r="O13" s="9" t="n"/>
       <c r="P13" s="9" t="n"/>
-      <c r="Q13" s="17" t="n"/>
-      <c r="R13" s="17" t="n"/>
-      <c r="S13" s="17" t="n"/>
+      <c r="Q13" s="9" t="n"/>
+      <c r="R13" s="9" t="n"/>
+      <c r="S13" s="9" t="n"/>
+      <c r="T13" s="9" t="n"/>
+      <c r="U13" s="9" t="n"/>
+      <c r="V13" s="9" t="n"/>
+      <c r="W13" s="9" t="n"/>
+      <c r="X13" s="17" t="n"/>
+      <c r="Y13" s="17" t="n"/>
+      <c r="Z13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
@@ -3475,9 +3750,16 @@
       <c r="N14" s="9" t="n"/>
       <c r="O14" s="9" t="n"/>
       <c r="P14" s="9" t="n"/>
-      <c r="Q14" s="17" t="n"/>
-      <c r="R14" s="17" t="n"/>
-      <c r="S14" s="17" t="n"/>
+      <c r="Q14" s="9" t="n"/>
+      <c r="R14" s="9" t="n"/>
+      <c r="S14" s="9" t="n"/>
+      <c r="T14" s="9" t="n"/>
+      <c r="U14" s="9" t="n"/>
+      <c r="V14" s="9" t="n"/>
+      <c r="W14" s="9" t="n"/>
+      <c r="X14" s="17" t="n"/>
+      <c r="Y14" s="17" t="n"/>
+      <c r="Z14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -3499,9 +3781,16 @@
       <c r="N15" s="9" t="n"/>
       <c r="O15" s="9" t="n"/>
       <c r="P15" s="9" t="n"/>
-      <c r="Q15" s="17" t="n"/>
-      <c r="R15" s="17" t="n"/>
-      <c r="S15" s="17" t="n"/>
+      <c r="Q15" s="9" t="n"/>
+      <c r="R15" s="9" t="n"/>
+      <c r="S15" s="9" t="n"/>
+      <c r="T15" s="9" t="n"/>
+      <c r="U15" s="9" t="n"/>
+      <c r="V15" s="9" t="n"/>
+      <c r="W15" s="9" t="n"/>
+      <c r="X15" s="17" t="n"/>
+      <c r="Y15" s="17" t="n"/>
+      <c r="Z15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -3523,9 +3812,16 @@
       <c r="N16" s="9" t="n"/>
       <c r="O16" s="9" t="n"/>
       <c r="P16" s="9" t="n"/>
-      <c r="Q16" s="17" t="n"/>
-      <c r="R16" s="17" t="n"/>
-      <c r="S16" s="17" t="n"/>
+      <c r="Q16" s="9" t="n"/>
+      <c r="R16" s="9" t="n"/>
+      <c r="S16" s="9" t="n"/>
+      <c r="T16" s="9" t="n"/>
+      <c r="U16" s="9" t="n"/>
+      <c r="V16" s="9" t="n"/>
+      <c r="W16" s="9" t="n"/>
+      <c r="X16" s="17" t="n"/>
+      <c r="Y16" s="17" t="n"/>
+      <c r="Z16" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3994,4 +4290,458 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Produto da semana (venda sem oferta, preço cheio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Novembro: semanas 1 e 2 só conteúdo (pós-Black). Venda contínua a partir da 3ª semana. Mentoria: 1 vez por mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Semana (início)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Tema da live</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Produto em destaque</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>2 peças de venda no feed (quais)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Story de venda todo dia?</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Bloco na newsletter?</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Vendas do produto na semana</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n"/>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n"/>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n"/>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="9" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="9" t="n"/>
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n"/>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="9" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n"/>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="n"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" s="9" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Nossos produtos</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Link de venda (com rastreio por canal)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Para quem é (1 linha)</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Temas de live ligados</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>[Pós 1]</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Pós</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>[Pós 2]</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Pós</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 1]</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 2]</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="9" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 3]</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 4]</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 5]</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 6]</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>[Curso 7]</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Curso</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Mentoria</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Mentoria</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pós,Curso,Mentoria,Só conteúdo"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Regras de venda nos stories (planilha aba 9 e roteiro)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Checklist do roteiro" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Calendário de captura" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Produto da semana" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Stories de venda" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -608,7 +609,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Toda semana tem venda. Feed: das 9 peças, 2 são de venda (caso real, depoimento, "isso a gente ensina na formação X"), umas 7 são conteúdo. Stories: todo dia pelo menos 1 story de venda, com link. Newsletter: sempre com o bloco da formação ligada ao tema. YouTube: link da formação na descrição.</t>
+          <t>Toda semana tem venda. Feed: das 9 peças, 2 são de venda (caso real, depoimento, "isso a gente ensina na formação X"), umas 7 são conteúdo. Stories: sequência de venda 3 vezes por semana (seg, qua, sex), seguindo as regras. Newsletter: sempre com o bloco da formação ligada ao tema. YouTube: link da formação na descrição.</t>
         </is>
       </c>
     </row>
@@ -648,7 +649,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>STORIES (todo dia)</t>
@@ -656,293 +657,305 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Ela planeja e roteiriza os stories da semana; quem aparece grava. Sequência diária de 5 a 8 stories: 1) bastidor ou rotina (gente real); 2) conteúdo rápido; 3) interação (enquete, caixinha, quiz); 4) prova (depoimento, print autorizado); 5) venda do produto da semana, com link.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
+          <t>Ela planeja e roteiriza os stories da semana; quem aparece grava. Todo dia: bastidor ou rotina, conteúdo rápido, interação (enquete, caixinha, quiz). Segunda, quarta e sexta: entra a sequência de venda (ver REGRAS DE VENDA NOS STORIES).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="135" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>REGRAS DE VENDA NOS STORIES</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>1) Venda nunca aparece sozinha: antes dela vêm pelo menos 2 stories do mesmo assunto (pergunta, caso, prova). 2) O link só entra no ÚLTIMO story da sequência. 3) No máximo 1 em cada 4 stories do dia é venda. 4) Pessoa vende melhor que arte: a venda é falada pelo Gabriel, pela Liliane ou por um aluno; a arte do produto só complementa. 5) Proibido: arte solta com "compre agora", urgência falsa ("últimas vagas" sem ser verdade), preço sem contexto. 6) Sequência completa de venda 3 vezes por semana (seg, qua, sex); nos outros dias, só conteúdo e interação, sem link de venda. Fim de semana: bastidor e leveza. 7) Quem responde enquete ou caixinha sobre o tema recebe DM: conversa vende mais que botão. Exemplos na aba 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>LINKS COM RASTREIO</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Cada canal tem link próprio com rastreio (UTM): bio, stories, newsletter, YouTube. Assim a Hotmart mostra de onde veio cada venda. A pessoa das automações monta. Sem isso, não dá para saber qual conteúdo vendeu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>VISÃO</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RESPONSÁVEL</t>
+          <t>VISÃO</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
+          <t>Reaquecer a base da FSA e deixá-la pronta para a próxima oferta. Instagram atrai e aquece; e-mail (newsletter) é a base que é nossa.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>QUEM APARECE</t>
+          <t>RESPONSÁVEL</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
+          <t>Uma pessoa: roteiros de reels, carrosséis, newsletter e criativo de captura. Ajuda na copy quando a Gisele pedir.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>QUEM APARECE</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Reels e carrosséis divididos entre o Gabriel de Carvalho e a professora Liliane. Ela distribui entre os dois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>O CENTRO DA SEMANA</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>A live semanal (aberta para toda a base). O tema da live vira a newsletter da semana. NÃO usar cortes da live como reels.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>ENTREGAS DA SEMANA</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>5 roteiros de reels + 4 carrosséis + 1 newsletter + YouTube (5 Shorts + 1 vídeo roteirizado + a live da semana). Um dos reels ou carrosséis é o criativo de captura ("comenta X e recebe Y").</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>YOUTUBE: SHORTS</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Os 5 reels da semana sobem também como Shorts no YouTube. Sem roteiro novo: é repostar, com título próprio para o YouTube.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>YOUTUBE: A LIVE DA SEMANA</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>A gravação da live sobe no YouTube toda semana. O trabalho dela: título forte (com a palavra que a pessoa buscaria no Google), capa com foto real e texto grande, descrição com o resumo, os momentos principais e o link da newsletter. Tempo: uns 30 minutos.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>YOUTUBE: VÍDEO ROTEIRIZADO</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>1 por semana, de 8 a 15 minutos, gravado pelo Gabriel ou pela Liliane. Usa o MESMO tema da newsletter da semana, mais aprofundado: a pesquisa já está feita, então o trabalho é o roteiro. Estrutura: gancho nos primeiros 30 segundos (a promessa do vídeo), desenvolvimento em blocos, caso prático, chamada para a newsletter.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="75" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26" ht="75" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>YOUTUBE: THUMB (CAPA)</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Toda thumb tem ROSTO, nunca só nome ou texto. Rosto grande, com expressão que chama atenção (surpresa, dúvida, preocupação, apontando). Foto real do professor, feita para a thumb. Até 4 palavras em letra grande, que completam o título sem repetir. Flecha ou círculo apontando para o elemento principal (o exame, o alimento, o número). Contraste forte. Testar se dá para ler no tamanho de celular.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>YOUTUBE: O PAPEL</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. O número que mostra se a thumb funciona é a TAXA DE CLIQUES (CTR) das impressões, no YouTube Studio.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+          <t>YOUTUBE: O PAPEL</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+          <t>Quem busca no YouTube quer conteúdo longo e pesquisa por assunto. Todo vídeo leva para a newsletter: link na descrição e no comentário fixado. O número que mostra se a thumb funciona é a TAXA DE CLIQUES (CTR) das impressões, no YouTube Studio.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>CRIATIVO DE CAPTURA (rodízio)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Semana 1: fica na DM (engajamento). Semana 2: DM pede o e-mail e o material chega por e-mail (base). Semana 3: carrossel com o tema da newsletter + convite "comenta NEWS". Semana 4: DM para e-mail com material de outra formação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>MATERIAL DE CAPTURA</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Sempre ligado a uma formação (exames, suplementação, hormonal, fertilidade, jejum, alergias). Nada genérico. Conteúdo técnico tirado do material da FSA (live ou aula), nunca de fonte de fora sem checar.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>ROTINA (D = dia da live)</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>D+1: transcrição (Descript) e rascunho da newsletter. SEXTA-FEIRA: manda numa mensagem só o PACOTE DA PRÓXIMA SEMANA (roteiros, carrosséis, newsletter, captura) + o RELATÓRIO DA SEMANA (aba 5 preenchida). Segunda a quinta: produz, publica e preenche o placar (aba 4). Newsletter: escrita a partir da live, enviada até 2 dias depois dela.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>IMAGENS (responsabilidade dela)</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Todo roteiro e carrossel sai com as imagens escolhidas, não só o texto. Imagem REAL, nunca de IA: professores, aulas, bastidores, prova (depoimentos e prints de alunos), e imagem daquilo que se está falando (o exame, o suplemento, o alimento). Muita imagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>BANCO DE IMAGENS</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ARTE DO CARROSSEL</t>
+          <t>BANCO DE IMAGENS</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
+          <t>Usar primeiro os bancos próprios da FSA (fotos e vídeos de professores, aulas, bastidores, prova). O Elements só para o que é genérico (alimento, laboratório, fundo).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AUTORIZAÇÃO DE IMAGEM</t>
+          <t>ARTE DO CARROSSEL</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
+          <t>A Claude monta o carrossel (skill carrossel FSA) a partir do texto e das fotos que ELA envia. Nenhuma imagem é gerada por IA: as fotos vêm sempre dos bancos da FSA ou do Elements.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>AUTORIZAÇÃO DE IMAGEM</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Depoimento e print de aluno só com autorização. Exame de paciente só sem nome, data de nascimento ou qualquer dado que identifique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>APROVAÇÃO</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Tudo passa pela Gisele antes de sair, em LOTE, uma vez por semana: na SEXTA, o pacote da semana seguinte. A primeira entrega é na segunda-feira, 26/10.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="45" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36" ht="45" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>PRIORIDADE SE O TEMPO APERTAR</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>1) Stories do dia (com o de venda)  2) Newsletter  3) As 2 peças de venda  4) Criativo de captura  5) Vídeo roteirizado do YouTube  6) Carrosséis e reels  7) Live e Shorts no YouTube</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>A META É RESULTADO</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>A META É RESULTADO</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Toda peça tem placar (aba 4). Gancho, retenção e conversão são medidos em cada reel. Não basta entregar: tem que superar a própria média.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>TODA SEMANA, 3 LINHAS</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>O que funcionou. O que não funcionou. O que vou testar na semana que vem. (aba 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="45" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>REGRAS QUE NÃO MUDAM</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>REGRAS QUE NÃO MUDAM</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Mesma mensagem da página de destino em toda peça de campanha. Fatos com fonte. Sem promessa de cura ou resultado. Respeitar as regras do conselho. Sem travessão. Português do Brasil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>BASE DE E-MAIL</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Reaquecer em ordem: semanas 1 e 2 só para quem abriu ou clicou nos últimos 6 meses; semana 3 campanha de reativação para os parados; depois tirar do envio quem não abre há 12 meses. Spam acima de 0,1%: parar e corrigir.</t>
         </is>
@@ -3848,7 +3861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4097,6 +4110,18 @@
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>STORIES DE VENDA: tem pelo menos 2 stories de contexto antes; o link está só no último; é falado por uma pessoa; não tem urgência falsa nem preço solto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>CAMPANHA: se fala de oferta, diz exatamente o que a página de destino diz (mesma frase, número, prazo).</t>
         </is>
@@ -4744,4 +4769,178 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sequência de venda nos stories (seg, qua, sex)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Função</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Exemplo (produto da semana: formação de exames)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Pergunta (interação)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Enquete: "Já atendeu paciente com o exame todo normal e cheio de sintomas?" Sim / Toda semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Conteúdo (pessoa falando)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Gabriel, 15 segundos: "Quando o exame vem normal, eu não paro na faixa de referência. Eu olho como um marcador conversa com o outro."</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Prova</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Print autorizado de aluna: "Depois da formação, nunca mais li hemograma do mesmo jeito." (sem dados de paciente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Venda, com link (só aqui)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Gabriel: "É isso que a gente ensina na Formação em Exames Laboratoriais. O link tá aqui." + figurinha de link com rastreio</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ERRADO</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Venda solta</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Arte do curso com "COMPRE AGORA" e o link, sem nenhum story antes sobre o assunto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>ERRADO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Urgência falsa</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>"Últimas vagas!" quando não é verdade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>ERRADO</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Venda todo dia</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Link de compra em todos os dias da semana: a audiência aprende a pular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Termômetro: se a taxa de saída no story de venda for bem maior que nos outros stories do dia, a venda está agressiva demais. Ajustar o contexto antes dela.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Stories: cardápio de formatos (vitrine, caixinha, quiz, bastidor, prova, escassez) e semana
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgesPtUiFaTyPjQzLX5smy
</commit_message>
<xml_diff>
--- a/fsa/conteudo-base/okr-conteudo-fsa.xlsx
+++ b/fsa/conteudo-base/okr-conteudo-fsa.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Checklist do roteiro" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Calendário de captura" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Produto da semana" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Stories de venda" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Stories (formatos)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -97,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,6 +124,9 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -657,19 +660,19 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Ela planeja e roteiriza os stories da semana; quem aparece grava. Todo dia: bastidor ou rotina, conteúdo rápido, interação (enquete, caixinha, quiz). Segunda, quarta e sexta: entra a sequência de venda (ver REGRAS DE VENDA NOS STORIES).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="135" customHeight="1">
+          <t>Ela planeja e roteiriza os stories da semana; quem aparece grava. Cada dia tem um formato diferente (aba 9). Venda na segunda (vitrine), quarta (consultoria na caixinha) e sexta (prova + objeção). Terça, quinta e fim de semana sem link de venda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>REGRAS DE VENDA NOS STORIES</t>
+          <t>STORIES: FORMATOS E REGRAS</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>1) Venda nunca aparece sozinha: antes dela vêm pelo menos 2 stories do mesmo assunto (pergunta, caso, prova). 2) O link só entra no ÚLTIMO story da sequência. 3) No máximo 1 em cada 4 stories do dia é venda. 4) Pessoa vende melhor que arte: a venda é falada pelo Gabriel, pela Liliane ou por um aluno; a arte do produto só complementa. 5) Proibido: arte solta com "compre agora", urgência falsa ("últimas vagas" sem ser verdade), preço sem contexto. 6) Sequência completa de venda 3 vezes por semana (seg, qua, sex); nos outros dias, só conteúdo e interação, sem link de venda. Fim de semana: bastidor e leveza. 7) Quem responde enquete ou caixinha sobre o tema recebe DM: conversa vende mais que botão. Exemplos na aba 9.</t>
+          <t>Ver a aba 9: cardápio de formatos, a semana e as regras de venda. Caixinha de perguntas no máximo 2 vezes por semana; nenhum formato todo dia.</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4114,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>STORIES DE VENDA: tem pelo menos 2 stories de contexto antes; o link está só no último; é falado por uma pessoa; não tem urgência falsa nem preço solto.</t>
+          <t>STORIES: o formato do dia é o da aba 9; antes do primeiro link tem pelo menos 2 stories de valor; a venda é falada por uma pessoa; sem urgência falsa nem preço solto.</t>
         </is>
       </c>
     </row>
@@ -4777,170 +4780,385 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sequência de venda nos stories (seg, qua, sex)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Story</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Função</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Exemplo (produto da semana: formação de exames)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Pergunta (interação)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Enquete: "Já atendeu paciente com o exame todo normal e cheio de sintomas?" Sim / Toda semana</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Conteúdo (pessoa falando)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Gabriel, 15 segundos: "Quando o exame vem normal, eu não paro na faixa de referência. Eu olho como um marcador conversa com o outro."</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Prova</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Print REAL de aluna, autorizado, falando do que mudou na leitura de exames. Nunca um depoimento inventado. Sem dados de paciente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Venda, com link (só aqui)</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Gabriel: "É isso que a gente ensina na Formação em Exames Laboratoriais. O link tá aqui." + figurinha de link com rastreio</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>ERRADO</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Venda solta</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Arte do curso com "COMPRE AGORA" e o link, sem nenhum story antes sobre o assunto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>ERRADO</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Urgência falsa</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>"Últimas vagas!" quando não é verdade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>ERRADO</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Venda todo dia</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Link de compra em todos os dias da semana: a audiência aprende a pular.</t>
+          <t>Cardápio de formatos de stories</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Variar é a regra: nenhum formato todo dia. Caixinha de perguntas no máximo 2 vezes por semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Como funciona</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Exemplo na FSA</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Frequência</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>VITRINE (venda)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Story 1: uma tese que o público reconhece + os 3 pilares + "vem ver como é por dentro". Stories 2 a 4: um pilar por story, com o professor em foto ou vídeo real de aula e 3 ou 4 ✅ do que se aprende. Último: o convite (link ou DM para o consultor). Pode abrir com uma enquete.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>"Chega uma hora em que o nutricionista precisa dominar mais do que o protocolo." Pilares da [formação da semana], cada um com o [professor] em aula. Convite: link ou "manda [PALAVRA] na DM".</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Segunda (produto da semana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>CONSULTORIA NA CAIXINHA (venda + leads)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Selfie sem produção convidando. Caixinha que QUALIFICA. Respostas curtas: 2 ou 3 ações + 1 frase de efeito. Uma pergunta vira convite ("isso a gente aprofunda na formação X", com link). Depois continua respondendo. Quem respondeu recebe DM do vendedor.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Gabriel: "Tua formação, há quanto tempo atende e o caso que mais te trava 👇". Responde como raciocínio clínico para profissionais, nunca prescrição para o paciente de alguém.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Quarta (1 vez; no máximo 2 por semana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>CASO COM QUIZ (engajamento)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Mostra um caso ou um exame (sem dados do paciente). Quiz ou enquete: "o que tu olharia primeiro?". No story seguinte, a resposta e o raciocínio. Sem link de venda.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Hemograma de um caso real anonimizado. Quiz com 3 opções. Gabriel ou Liliane explicam a resposta em 15 segundos.</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>BASTIDOR (conexão)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Gente real e rotina: aula sendo gravada, equipe, professor preparando a live, aluno na sala. Leve, sem venda. Uma enquete divertida ajuda.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>"Hoje é dia de gravação da aula de [tema]", com vídeo curto do estúdio ou da sala.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Quinta e fim de semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>PROVA + OBJEÇÃO (venda)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Depoimento ou print REAL de aluno (autorizado), resultado de turma, e uma objeção respondida pelo Gabriel ("não tenho tempo", "é caro"). Fecha com convite para o consultor.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Print real de aluna + Gabriel respondendo "Gabriel, eu não tenho tempo" + "manda [PALAVRA] na DM que o consultor te ajuda a escolher".</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>ESCASSEZ COM 2ª CHANCE (venda)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Aviso antes, abertura, "últimas vagas", fechou, nova porta (lista de espera). Print da página real como prova. Story repetido só com o link.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Turma de pós abrindo: "as inscrições da turma [X] abrem dia [data]. Entra na lista e fala antes com o consultor."</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>SÓ quando houver turma ou prazo de verdade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>ENQUETE DE OPINIÃO (engajamento)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Uma pergunta que divide opiniões do público profissional. Quem vota recebe DM com um conteúdo sobre o tema.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>"Ferritina baixa com hemoglobina normal: tu suplementa?" Sim / Depende</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Qualquer dia, como abertura</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Termômetro: se a taxa de saída no story de venda for bem maior que nos outros stories do dia, a venda está agressiva demais. Ajustar o contexto antes dela.</t>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>A SEMANA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Vitrine do produto da semana (venda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Caso com quiz (sem link de venda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Quarta</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Consultoria na caixinha (venda + leads para o vendedor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bastidor (sem link de venda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Prova + objeção (venda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sábado e domingo</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bastidor e leveza</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>REGRAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Antes do primeiro link, sempre tem valor (pelo menos 2 stories do assunto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Numa sequência longa, o link pode aparecer no meio e se repetir, desde que entre um e outro tenha mais valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Pessoa vende melhor que arte: a venda é falada pelo Gabriel, pela Liliane ou por um aluno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Proibido: arte solta com "compre agora", urgência falsa, preço sem contexto, depoimento inventado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Para pós e mentoria, o convite é para conversar com o consultor (DM ou WhatsApp), não para um formulário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Quem responde enquete, quiz ou caixinha sobre o tema recebe DM. Conversa vende mais que botão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>7.</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Termômetro: se muita gente sai justo no story de venda, a venda está agressiva demais.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>